<commit_message>
Renombrar funciones y variables, simplificar comentarios y regenerar resultados
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resultados_tarea3.xlsx
+++ b/resultados_tarea3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Resumen" sheetId="1" r:id="rId1"/>
     <sheet name="Iteraciones" sheetId="2" r:id="rId2"/>
     <sheet name="Columnas generadas" sheetId="3" r:id="rId3"/>
-    <sheet name="Solucion LP" sheetId="4" r:id="rId4"/>
+    <sheet name="Solucion relajada" sheetId="4" r:id="rId4"/>
     <sheet name="Solucion entera" sheetId="5" r:id="rId5"/>
     <sheet name="Turnos por dia" sheetId="6" r:id="rId6"/>
     <sheet name="Requerimiento" sheetId="7" r:id="rId7"/>
@@ -37,22 +37,22 @@
     <t>Iteraciones</t>
   </si>
   <si>
-    <t>Costo RMP (LP)</t>
-  </si>
-  <si>
-    <t>Costo IMP (entero)</t>
-  </si>
-  <si>
-    <t>ceil(z_LP)</t>
-  </si>
-  <si>
-    <t>Brecha % vs z_LP</t>
-  </si>
-  <si>
-    <t>Tripulaciones (entero)</t>
-  </si>
-  <si>
-    <t>Cota inferior tripulaciones (fin de semana)</t>
+    <t>Costo relajado</t>
+  </si>
+  <si>
+    <t>Costo entero</t>
+  </si>
+  <si>
+    <t>Cota inferior redondeada</t>
+  </si>
+  <si>
+    <t>Brecha %</t>
+  </si>
+  <si>
+    <t>Tripulaciones</t>
+  </si>
+  <si>
+    <t>Minimo de tripulaciones por fin de semana</t>
   </si>
   <si>
     <t>Exceso de cobertura</t>
@@ -61,7 +61,7 @@
     <t>iteracion</t>
   </si>
   <si>
-    <t>FO_RMP</t>
+    <t>FO_maestro</t>
   </si>
   <si>
     <t>costo_reducido_min</t>
@@ -82,202 +82,202 @@
     <t>turno</t>
   </si>
   <si>
-    <t>Lun 06-14 | Mar 06-14 | Mié ---- | Jue 06-14 | Vie 06-14 | Sáb ---- | Dom 06-14</t>
-  </si>
-  <si>
-    <t>Lun 14-22 | Mar 14-22 | Mié ---- | Jue 14-22 | Vie 14-22 | Sáb ---- | Dom 14-22</t>
-  </si>
-  <si>
-    <t>Lun 00-08 | Mar 00-08 | Mié ---- | Jue 00-08 | Vie 00-08 | Sáb ---- | Dom 00-08</t>
-  </si>
-  <si>
-    <t>Lun 16-24 | Mar ---- | Mié 06-14 | Jue ---- | Vie 16-24 | Sáb 06-14 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun 06-14 | Mar ---- | Mié 14-22 | Jue 16-24 | Vie ---- | Sáb 14-22 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun ---- | Mar 16-24 | Mié 00-08 | Jue ---- | Vie 06-14 | Sáb 00-08 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun 06-14 | Mar ---- | Mié 16-24 | Jue 02-10 | Vie ---- | Sáb ---- | Dom 16-24</t>
-  </si>
-  <si>
-    <t>Lun 06-14 | Mar 00-08 | Mié ---- | Jue ---- | Vie 08-16 | Sáb 16-24 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun 08-16 | Mar 06-14 | Mié ---- | Jue 06-14 | Vie ---- | Sáb 08-16 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun 06-14 | Mar ---- | Mié ---- | Jue 14-22 | Vie 12-20 | Sáb ---- | Dom 02-10</t>
-  </si>
-  <si>
-    <t>Lun 06-14 | Mar ---- | Mié ---- | Jue 14-22 | Vie 14-22 | Sáb ---- | Dom 00-08</t>
-  </si>
-  <si>
-    <t>Lun 06-14 | Mar ---- | Mié ---- | Jue 14-22 | Vie 02-10 | Sáb ---- | Dom 08-16</t>
-  </si>
-  <si>
-    <t>Lun 04-12 | Mar 08-16 | Mié ---- | Jue 16-24 | Vie ---- | Sáb 00-08 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun 02-10 | Mar ---- | Mié 08-16 | Jue ---- | Vie 12-20 | Sáb ---- | Dom 16-24</t>
-  </si>
-  <si>
-    <t>Lun 00-08 | Mar 12-20 | Mié ---- | Jue 16-24 | Vie 14-22 | Sáb ---- | Dom 06-14</t>
-  </si>
-  <si>
-    <t>Lun 14-22 | Mar ---- | Mié 08-16 | Jue ---- | Vie 00-08 | Sáb ---- | Dom 06-14</t>
-  </si>
-  <si>
-    <t>Lun 16-24 | Mar ---- | Mié 08-16 | Jue 06-14 | Vie ---- | Sáb ---- | Dom 08-16</t>
-  </si>
-  <si>
-    <t>Lun ---- | Mar 12-20 | Mié ---- | Jue 00-08 | Vie 14-22 | Sáb ---- | Dom 06-14</t>
-  </si>
-  <si>
-    <t>Lun 00-08 | Mar 12-20 | Mié ---- | Jue ---- | Vie 16-24 | Sáb ---- | Dom 00-08</t>
-  </si>
-  <si>
-    <t>Lun 00-08 | Mar ---- | Mié ---- | Jue 14-22 | Vie 00-08 | Sáb ---- | Dom 14-22</t>
-  </si>
-  <si>
-    <t>Lun 00-08 | Mar 16-24 | Mié ---- | Jue ---- | Vie 00-08 | Sáb ---- | Dom 16-24</t>
-  </si>
-  <si>
-    <t>Lun 02-10 | Mar ---- | Mié ---- | Jue 02-10 | Vie 02-10 | Sáb ---- | Dom 02-10</t>
-  </si>
-  <si>
-    <t>Lun 00-08 | Mar ---- | Mié 10-18 | Jue ---- | Vie 14-22 | Sáb 00-08 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun 00-08 | Mar ---- | Mié 00-08 | Jue 02-10 | Vie ---- | Sáb 16-24 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun 06-14 | Mar ---- | Mié ---- | Jue 00-08 | Vie 16-24 | Sáb ---- | Dom 16-24</t>
-  </si>
-  <si>
-    <t>Lun 16-24 | Mar 12-20 | Mié ---- | Jue ---- | Vie 02-10 | Sáb 16-24 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun 02-10 | Mar 16-24 | Mié ---- | Jue ---- | Vie 16-24 | Sáb ---- | Dom 06-14</t>
-  </si>
-  <si>
-    <t>Lun ---- | Mar 12-20 | Mié 16-24 | Jue ---- | Vie 16-24 | Sáb 16-24 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun 00-08 | Mar ---- | Mié 00-08 | Jue 14-22 | Vie ---- | Sáb ---- | Dom 06-14</t>
-  </si>
-  <si>
-    <t>Lun 06-14 | Mar ---- | Mié ---- | Jue 02-10 | Vie 00-08 | Sáb ---- | Dom 06-14</t>
-  </si>
-  <si>
-    <t>Lun 06-14 | Mar ---- | Mié 00-08 | Jue ---- | Vie 14-22 | Sáb ---- | Dom 14-22</t>
-  </si>
-  <si>
-    <t>Lun ---- | Mar 16-24 | Mié ---- | Jue 16-24 | Vie 12-20 | Sáb ---- | Dom 06-14</t>
-  </si>
-  <si>
-    <t>Lun ---- | Mar 12-20 | Mié ---- | Jue 14-22 | Vie 06-14 | Sáb ---- | Dom 16-24</t>
-  </si>
-  <si>
-    <t>Lun ---- | Mar 00-08 | Mié 16-24 | Jue ---- | Vie 02-10 | Sáb ---- | Dom 06-14</t>
-  </si>
-  <si>
-    <t>Lun 06-14 | Mar ---- | Mié 06-14 | Jue 16-24 | Vie ---- | Sáb ---- | Dom 02-10</t>
-  </si>
-  <si>
-    <t>Lun 02-10 | Mar ---- | Mié 16-24 | Jue 00-08 | Vie ---- | Sáb 00-08 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun 06-14 | Mar ---- | Mié 06-14 | Jue 16-24 | Vie ---- | Sáb 00-08 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun 04-12 | Mar ---- | Mié ---- | Jue 06-14 | Vie 12-20 | Sáb ---- | Dom 06-14</t>
-  </si>
-  <si>
-    <t>Lun 06-14 | Mar ---- | Mié ---- | Jue 06-14 | Vie 06-14 | Sáb ---- | Dom 06-14</t>
-  </si>
-  <si>
-    <t>Lun 04-12 | Mar 00-08 | Mié ---- | Jue 00-08 | Vie ---- | Sáb ---- | Dom 02-10</t>
-  </si>
-  <si>
-    <t>Lun 00-08 | Mar ---- | Mié 00-08 | Jue ---- | Vie 00-08 | Sáb 00-08 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun 14-22 | Mar ---- | Mié ---- | Jue 02-10 | Vie 12-20 | Sáb ---- | Dom 14-22</t>
-  </si>
-  <si>
-    <t>Lun 14-22 | Mar 12-20 | Mié ---- | Jue ---- | Vie 14-22 | Sáb 00-08 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun 14-22 | Mar ---- | Mié 16-24 | Jue 00-08 | Vie ---- | Sáb 00-08 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun ---- | Mar 12-20 | Mié 08-16 | Jue ---- | Vie 12-20 | Sáb 06-14 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun 04-12 | Mar ---- | Mié 10-18 | Jue ---- | Vie 00-08 | Sáb ---- | Dom 00-08</t>
-  </si>
-  <si>
-    <t>Lun ---- | Mar 12-20 | Mié 00-08 | Jue ---- | Vie 00-08 | Sáb 06-14 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun ---- | Mar 06-14 | Mié 06-14 | Jue ---- | Vie 00-08 | Sáb 16-24 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun ---- | Mar 00-08 | Mié ---- | Jue 02-10 | Vie 02-10 | Sáb ---- | Dom 00-08</t>
-  </si>
-  <si>
-    <t>Lun 04-12 | Mar 00-08 | Mié ---- | Jue 00-08 | Vie ---- | Sáb 06-14 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun 00-08 | Mar 06-14 | Mié ---- | Jue 00-08 | Vie ---- | Sáb 06-14 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun 04-12 | Mar ---- | Mié 08-16 | Jue ---- | Vie 06-14 | Sáb 06-14 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun 14-22 | Mar 00-08 | Mié ---- | Jue ---- | Vie 06-14 | Sáb 08-16 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun 00-08 | Mar 00-08 | Mié ---- | Jue ---- | Vie 14-22 | Sáb ---- | Dom 08-16</t>
-  </si>
-  <si>
-    <t>Lun 06-14 | Mar ---- | Mié 16-24 | Jue ---- | Vie 02-10 | Sáb ---- | Dom 14-22</t>
-  </si>
-  <si>
-    <t>Lun ---- | Mar 16-24 | Mié 08-16 | Jue ---- | Vie 06-14 | Sáb ---- | Dom 14-22</t>
-  </si>
-  <si>
-    <t>Lun 00-08 | Mar 06-14 | Mié ---- | Jue ---- | Vie 06-14 | Sáb ---- | Dom 00-08</t>
-  </si>
-  <si>
-    <t>Lun ---- | Mar 00-08 | Mié 08-16 | Jue ---- | Vie 14-22 | Sáb ---- | Dom 02-10</t>
-  </si>
-  <si>
-    <t>Lun ---- | Mar 06-14 | Mié 06-14 | Jue ---- | Vie 06-14 | Sáb 16-24 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun 16-24 | Mar 00-08 | Mié ---- | Jue ---- | Vie 00-08 | Sáb ---- | Dom 16-24</t>
-  </si>
-  <si>
-    <t>Lun 00-08 | Mar 00-08 | Mié ---- | Jue 14-22 | Vie ---- | Sáb 00-08 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun ---- | Mar 00-08 | Mié 08-16 | Jue ---- | Vie 00-08 | Sáb 06-14 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun 02-10 | Mar 16-24 | Mié ---- | Jue 02-10 | Vie ---- | Sáb 06-14 | Dom ----</t>
-  </si>
-  <si>
-    <t>Lun 08-16 | Mar 00-08 | Mié ---- | Jue 00-08 | Vie ---- | Sáb ---- | Dom 00-08</t>
-  </si>
-  <si>
-    <t>Lun 06-14 | Mar 16-24 | Mié ---- | Jue 06-14 | Vie ---- | Sáb 06-14 | Dom ----</t>
-  </si>
-  <si>
-    <t>x_LP</t>
+    <t>Lun 06-14 | Mar 06-14 | Mié Libre | Jue 06-14 | Vie 06-14 | Sáb Libre | Dom 06-14</t>
+  </si>
+  <si>
+    <t>Lun 14-22 | Mar 14-22 | Mié Libre | Jue 14-22 | Vie 14-22 | Sáb Libre | Dom 14-22</t>
+  </si>
+  <si>
+    <t>Lun 00-08 | Mar 00-08 | Mié Libre | Jue 00-08 | Vie 00-08 | Sáb Libre | Dom 00-08</t>
+  </si>
+  <si>
+    <t>Lun 16-24 | Mar Libre | Mié 06-14 | Jue Libre | Vie 16-24 | Sáb 06-14 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun 06-14 | Mar Libre | Mié 14-22 | Jue 16-24 | Vie Libre | Sáb 14-22 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun Libre | Mar 16-24 | Mié 00-08 | Jue Libre | Vie 06-14 | Sáb 00-08 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun 06-14 | Mar Libre | Mié 16-24 | Jue 02-10 | Vie Libre | Sáb Libre | Dom 16-24</t>
+  </si>
+  <si>
+    <t>Lun 06-14 | Mar 00-08 | Mié Libre | Jue Libre | Vie 08-16 | Sáb 16-24 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun 08-16 | Mar 06-14 | Mié Libre | Jue 06-14 | Vie Libre | Sáb 08-16 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun 06-14 | Mar Libre | Mié Libre | Jue 14-22 | Vie 12-20 | Sáb Libre | Dom 02-10</t>
+  </si>
+  <si>
+    <t>Lun 06-14 | Mar Libre | Mié Libre | Jue 14-22 | Vie 14-22 | Sáb Libre | Dom 00-08</t>
+  </si>
+  <si>
+    <t>Lun 06-14 | Mar Libre | Mié Libre | Jue 14-22 | Vie 02-10 | Sáb Libre | Dom 08-16</t>
+  </si>
+  <si>
+    <t>Lun 04-12 | Mar 08-16 | Mié Libre | Jue 16-24 | Vie Libre | Sáb 00-08 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun 02-10 | Mar Libre | Mié 08-16 | Jue Libre | Vie 12-20 | Sáb Libre | Dom 16-24</t>
+  </si>
+  <si>
+    <t>Lun 00-08 | Mar 12-20 | Mié Libre | Jue 16-24 | Vie 14-22 | Sáb Libre | Dom 06-14</t>
+  </si>
+  <si>
+    <t>Lun 14-22 | Mar Libre | Mié 08-16 | Jue Libre | Vie 00-08 | Sáb Libre | Dom 06-14</t>
+  </si>
+  <si>
+    <t>Lun 16-24 | Mar Libre | Mié 08-16 | Jue 06-14 | Vie Libre | Sáb Libre | Dom 08-16</t>
+  </si>
+  <si>
+    <t>Lun Libre | Mar 12-20 | Mié Libre | Jue 00-08 | Vie 14-22 | Sáb Libre | Dom 06-14</t>
+  </si>
+  <si>
+    <t>Lun 00-08 | Mar 12-20 | Mié Libre | Jue Libre | Vie 16-24 | Sáb Libre | Dom 00-08</t>
+  </si>
+  <si>
+    <t>Lun 00-08 | Mar Libre | Mié Libre | Jue 14-22 | Vie 00-08 | Sáb Libre | Dom 14-22</t>
+  </si>
+  <si>
+    <t>Lun 00-08 | Mar 16-24 | Mié Libre | Jue Libre | Vie 00-08 | Sáb Libre | Dom 16-24</t>
+  </si>
+  <si>
+    <t>Lun 02-10 | Mar Libre | Mié Libre | Jue 02-10 | Vie 02-10 | Sáb Libre | Dom 02-10</t>
+  </si>
+  <si>
+    <t>Lun 00-08 | Mar Libre | Mié 10-18 | Jue Libre | Vie 14-22 | Sáb 00-08 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun 00-08 | Mar Libre | Mié 00-08 | Jue 02-10 | Vie Libre | Sáb 16-24 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun 06-14 | Mar Libre | Mié Libre | Jue 00-08 | Vie 16-24 | Sáb Libre | Dom 16-24</t>
+  </si>
+  <si>
+    <t>Lun 16-24 | Mar 12-20 | Mié Libre | Jue Libre | Vie 02-10 | Sáb 16-24 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun 02-10 | Mar 16-24 | Mié Libre | Jue Libre | Vie 16-24 | Sáb Libre | Dom 06-14</t>
+  </si>
+  <si>
+    <t>Lun Libre | Mar 12-20 | Mié 16-24 | Jue Libre | Vie 16-24 | Sáb 16-24 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun 00-08 | Mar Libre | Mié 00-08 | Jue 14-22 | Vie Libre | Sáb Libre | Dom 06-14</t>
+  </si>
+  <si>
+    <t>Lun 06-14 | Mar Libre | Mié Libre | Jue 02-10 | Vie 00-08 | Sáb Libre | Dom 06-14</t>
+  </si>
+  <si>
+    <t>Lun 06-14 | Mar Libre | Mié 00-08 | Jue Libre | Vie 14-22 | Sáb Libre | Dom 14-22</t>
+  </si>
+  <si>
+    <t>Lun Libre | Mar 16-24 | Mié Libre | Jue 16-24 | Vie 12-20 | Sáb Libre | Dom 06-14</t>
+  </si>
+  <si>
+    <t>Lun Libre | Mar 12-20 | Mié Libre | Jue 14-22 | Vie 06-14 | Sáb Libre | Dom 16-24</t>
+  </si>
+  <si>
+    <t>Lun Libre | Mar 00-08 | Mié 16-24 | Jue Libre | Vie 02-10 | Sáb Libre | Dom 06-14</t>
+  </si>
+  <si>
+    <t>Lun 06-14 | Mar Libre | Mié 06-14 | Jue 16-24 | Vie Libre | Sáb Libre | Dom 02-10</t>
+  </si>
+  <si>
+    <t>Lun 02-10 | Mar Libre | Mié 16-24 | Jue 00-08 | Vie Libre | Sáb 00-08 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun 06-14 | Mar Libre | Mié 06-14 | Jue 16-24 | Vie Libre | Sáb 00-08 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun 04-12 | Mar Libre | Mié Libre | Jue 06-14 | Vie 12-20 | Sáb Libre | Dom 06-14</t>
+  </si>
+  <si>
+    <t>Lun 06-14 | Mar Libre | Mié Libre | Jue 06-14 | Vie 06-14 | Sáb Libre | Dom 06-14</t>
+  </si>
+  <si>
+    <t>Lun 04-12 | Mar 00-08 | Mié Libre | Jue 00-08 | Vie Libre | Sáb Libre | Dom 02-10</t>
+  </si>
+  <si>
+    <t>Lun 00-08 | Mar Libre | Mié 00-08 | Jue Libre | Vie 00-08 | Sáb 00-08 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun 14-22 | Mar Libre | Mié Libre | Jue 02-10 | Vie 12-20 | Sáb Libre | Dom 14-22</t>
+  </si>
+  <si>
+    <t>Lun 14-22 | Mar 12-20 | Mié Libre | Jue Libre | Vie 14-22 | Sáb 00-08 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun 14-22 | Mar Libre | Mié 16-24 | Jue 00-08 | Vie Libre | Sáb 00-08 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun Libre | Mar 12-20 | Mié 08-16 | Jue Libre | Vie 12-20 | Sáb 06-14 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun 04-12 | Mar Libre | Mié 10-18 | Jue Libre | Vie 00-08 | Sáb Libre | Dom 00-08</t>
+  </si>
+  <si>
+    <t>Lun Libre | Mar 12-20 | Mié 00-08 | Jue Libre | Vie 00-08 | Sáb 06-14 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun Libre | Mar 06-14 | Mié 06-14 | Jue Libre | Vie 00-08 | Sáb 16-24 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun Libre | Mar 00-08 | Mié Libre | Jue 02-10 | Vie 02-10 | Sáb Libre | Dom 00-08</t>
+  </si>
+  <si>
+    <t>Lun 04-12 | Mar 00-08 | Mié Libre | Jue 00-08 | Vie Libre | Sáb 06-14 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun 00-08 | Mar 06-14 | Mié Libre | Jue 00-08 | Vie Libre | Sáb 06-14 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun 04-12 | Mar Libre | Mié 08-16 | Jue Libre | Vie 06-14 | Sáb 06-14 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun 14-22 | Mar 00-08 | Mié Libre | Jue Libre | Vie 06-14 | Sáb 08-16 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun 00-08 | Mar 00-08 | Mié Libre | Jue Libre | Vie 14-22 | Sáb Libre | Dom 08-16</t>
+  </si>
+  <si>
+    <t>Lun 06-14 | Mar Libre | Mié 16-24 | Jue Libre | Vie 02-10 | Sáb Libre | Dom 14-22</t>
+  </si>
+  <si>
+    <t>Lun Libre | Mar 16-24 | Mié 08-16 | Jue Libre | Vie 06-14 | Sáb Libre | Dom 14-22</t>
+  </si>
+  <si>
+    <t>Lun 00-08 | Mar 06-14 | Mié Libre | Jue Libre | Vie 06-14 | Sáb Libre | Dom 00-08</t>
+  </si>
+  <si>
+    <t>Lun Libre | Mar 00-08 | Mié 08-16 | Jue Libre | Vie 14-22 | Sáb Libre | Dom 02-10</t>
+  </si>
+  <si>
+    <t>Lun Libre | Mar 06-14 | Mié 06-14 | Jue Libre | Vie 06-14 | Sáb 16-24 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun 16-24 | Mar 00-08 | Mié Libre | Jue Libre | Vie 00-08 | Sáb Libre | Dom 16-24</t>
+  </si>
+  <si>
+    <t>Lun 00-08 | Mar 00-08 | Mié Libre | Jue 14-22 | Vie Libre | Sáb 00-08 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun Libre | Mar 00-08 | Mié 08-16 | Jue Libre | Vie 00-08 | Sáb 06-14 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun 02-10 | Mar 16-24 | Mié Libre | Jue 02-10 | Vie Libre | Sáb 06-14 | Dom Libre</t>
+  </si>
+  <si>
+    <t>Lun 08-16 | Mar 00-08 | Mié Libre | Jue 00-08 | Vie Libre | Sáb Libre | Dom 00-08</t>
+  </si>
+  <si>
+    <t>Lun 06-14 | Mar 16-24 | Mié Libre | Jue 06-14 | Vie Libre | Sáb 06-14 | Dom Libre</t>
+  </si>
+  <si>
+    <t>x_relajado</t>
   </si>
   <si>
     <t>Lunes</t>
@@ -337,7 +337,7 @@
     <t>dia</t>
   </si>
   <si>
-    <t>min_turnos_necesarios</t>
+    <t>minimo_turnos</t>
   </si>
   <si>
     <t>tripulaciones_asignadas</t>
@@ -4070,28 +4070,28 @@
         <v>17</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>102</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -4104,29 +4104,29 @@
       <c r="C2">
         <v>1164</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E2" t="s">
+        <v>93</v>
+      </c>
+      <c r="F2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H2" t="s">
+        <v>93</v>
+      </c>
+      <c r="I2" t="s">
+        <v>94</v>
+      </c>
+      <c r="J2" t="s">
+        <v>92</v>
+      </c>
+      <c r="K2">
         <v>89628</v>
-      </c>
-      <c r="E2" t="s">
-        <v>92</v>
-      </c>
-      <c r="F2" t="s">
-        <v>93</v>
-      </c>
-      <c r="G2" t="s">
-        <v>93</v>
-      </c>
-      <c r="H2" t="s">
-        <v>92</v>
-      </c>
-      <c r="I2" t="s">
-        <v>93</v>
-      </c>
-      <c r="J2" t="s">
-        <v>94</v>
-      </c>
-      <c r="K2" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -4139,29 +4139,29 @@
       <c r="C3">
         <v>1128</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="s">
+        <v>93</v>
+      </c>
+      <c r="E3" t="s">
+        <v>92</v>
+      </c>
+      <c r="F3" t="s">
+        <v>92</v>
+      </c>
+      <c r="G3" t="s">
+        <v>93</v>
+      </c>
+      <c r="H3" t="s">
+        <v>93</v>
+      </c>
+      <c r="I3" t="s">
+        <v>92</v>
+      </c>
+      <c r="J3" t="s">
+        <v>93</v>
+      </c>
+      <c r="K3">
         <v>56400</v>
-      </c>
-      <c r="E3" t="s">
-        <v>93</v>
-      </c>
-      <c r="F3" t="s">
-        <v>92</v>
-      </c>
-      <c r="G3" t="s">
-        <v>92</v>
-      </c>
-      <c r="H3" t="s">
-        <v>93</v>
-      </c>
-      <c r="I3" t="s">
-        <v>93</v>
-      </c>
-      <c r="J3" t="s">
-        <v>92</v>
-      </c>
-      <c r="K3" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -4174,29 +4174,29 @@
       <c r="C4">
         <v>1455</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="s">
+        <v>93</v>
+      </c>
+      <c r="E4" t="s">
+        <v>92</v>
+      </c>
+      <c r="F4" t="s">
+        <v>94</v>
+      </c>
+      <c r="G4" t="s">
+        <v>99</v>
+      </c>
+      <c r="H4" t="s">
+        <v>92</v>
+      </c>
+      <c r="I4" t="s">
+        <v>92</v>
+      </c>
+      <c r="J4" t="s">
+        <v>94</v>
+      </c>
+      <c r="K4">
         <v>72750</v>
-      </c>
-      <c r="E4" t="s">
-        <v>93</v>
-      </c>
-      <c r="F4" t="s">
-        <v>92</v>
-      </c>
-      <c r="G4" t="s">
-        <v>94</v>
-      </c>
-      <c r="H4" t="s">
-        <v>99</v>
-      </c>
-      <c r="I4" t="s">
-        <v>92</v>
-      </c>
-      <c r="J4" t="s">
-        <v>92</v>
-      </c>
-      <c r="K4" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -4209,29 +4209,29 @@
       <c r="C5">
         <v>1368</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="s">
+        <v>92</v>
+      </c>
+      <c r="E5" t="s">
+        <v>94</v>
+      </c>
+      <c r="F5" t="s">
+        <v>96</v>
+      </c>
+      <c r="G5" t="s">
+        <v>92</v>
+      </c>
+      <c r="H5" t="s">
+        <v>93</v>
+      </c>
+      <c r="I5" t="s">
+        <v>96</v>
+      </c>
+      <c r="J5" t="s">
+        <v>92</v>
+      </c>
+      <c r="K5">
         <v>46512</v>
-      </c>
-      <c r="E5" t="s">
-        <v>92</v>
-      </c>
-      <c r="F5" t="s">
-        <v>94</v>
-      </c>
-      <c r="G5" t="s">
-        <v>96</v>
-      </c>
-      <c r="H5" t="s">
-        <v>92</v>
-      </c>
-      <c r="I5" t="s">
-        <v>93</v>
-      </c>
-      <c r="J5" t="s">
-        <v>96</v>
-      </c>
-      <c r="K5" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -4244,29 +4244,29 @@
       <c r="C6">
         <v>1266</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="s">
+        <v>93</v>
+      </c>
+      <c r="E6" t="s">
+        <v>92</v>
+      </c>
+      <c r="F6" t="s">
+        <v>93</v>
+      </c>
+      <c r="G6" t="s">
+        <v>94</v>
+      </c>
+      <c r="H6" t="s">
+        <v>92</v>
+      </c>
+      <c r="I6" t="s">
+        <v>96</v>
+      </c>
+      <c r="J6" t="s">
+        <v>92</v>
+      </c>
+      <c r="K6">
         <v>40512</v>
-      </c>
-      <c r="E6" t="s">
-        <v>93</v>
-      </c>
-      <c r="F6" t="s">
-        <v>92</v>
-      </c>
-      <c r="G6" t="s">
-        <v>93</v>
-      </c>
-      <c r="H6" t="s">
-        <v>94</v>
-      </c>
-      <c r="I6" t="s">
-        <v>92</v>
-      </c>
-      <c r="J6" t="s">
-        <v>96</v>
-      </c>
-      <c r="K6" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -4279,29 +4279,29 @@
       <c r="C7">
         <v>1426</v>
       </c>
-      <c r="D7">
-        <v>42780</v>
+      <c r="D7" t="s">
+        <v>93</v>
       </c>
       <c r="E7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F7" t="s">
         <v>92</v>
       </c>
       <c r="G7" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="H7" t="s">
         <v>97</v>
       </c>
       <c r="I7" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="J7" t="s">
-        <v>92</v>
-      </c>
-      <c r="K7" t="s">
-        <v>96</v>
+        <v>96</v>
+      </c>
+      <c r="K7">
+        <v>42780</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -4314,29 +4314,29 @@
       <c r="C8">
         <v>1068</v>
       </c>
-      <c r="D8">
+      <c r="D8" t="s">
+        <v>95</v>
+      </c>
+      <c r="E8" t="s">
+        <v>93</v>
+      </c>
+      <c r="F8" t="s">
+        <v>92</v>
+      </c>
+      <c r="G8" t="s">
+        <v>93</v>
+      </c>
+      <c r="H8" t="s">
+        <v>92</v>
+      </c>
+      <c r="I8" t="s">
+        <v>95</v>
+      </c>
+      <c r="J8" t="s">
+        <v>92</v>
+      </c>
+      <c r="K8">
         <v>27768</v>
-      </c>
-      <c r="E8" t="s">
-        <v>95</v>
-      </c>
-      <c r="F8" t="s">
-        <v>93</v>
-      </c>
-      <c r="G8" t="s">
-        <v>92</v>
-      </c>
-      <c r="H8" t="s">
-        <v>93</v>
-      </c>
-      <c r="I8" t="s">
-        <v>92</v>
-      </c>
-      <c r="J8" t="s">
-        <v>95</v>
-      </c>
-      <c r="K8" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -4349,29 +4349,29 @@
       <c r="C9">
         <v>1272</v>
       </c>
-      <c r="D9">
+      <c r="D9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E9" t="s">
+        <v>92</v>
+      </c>
+      <c r="F9" t="s">
+        <v>93</v>
+      </c>
+      <c r="G9" t="s">
+        <v>92</v>
+      </c>
+      <c r="H9" t="s">
+        <v>94</v>
+      </c>
+      <c r="I9" t="s">
+        <v>93</v>
+      </c>
+      <c r="J9" t="s">
+        <v>92</v>
+      </c>
+      <c r="K9">
         <v>22896</v>
-      </c>
-      <c r="E9" t="s">
-        <v>94</v>
-      </c>
-      <c r="F9" t="s">
-        <v>92</v>
-      </c>
-      <c r="G9" t="s">
-        <v>93</v>
-      </c>
-      <c r="H9" t="s">
-        <v>92</v>
-      </c>
-      <c r="I9" t="s">
-        <v>94</v>
-      </c>
-      <c r="J9" t="s">
-        <v>93</v>
-      </c>
-      <c r="K9" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -4384,29 +4384,29 @@
       <c r="C10">
         <v>1591</v>
       </c>
-      <c r="D10">
+      <c r="D10" t="s">
+        <v>94</v>
+      </c>
+      <c r="E10" t="s">
+        <v>96</v>
+      </c>
+      <c r="F10" t="s">
+        <v>92</v>
+      </c>
+      <c r="G10" t="s">
+        <v>92</v>
+      </c>
+      <c r="H10" t="s">
+        <v>96</v>
+      </c>
+      <c r="I10" t="s">
+        <v>92</v>
+      </c>
+      <c r="J10" t="s">
+        <v>94</v>
+      </c>
+      <c r="K10">
         <v>27047</v>
-      </c>
-      <c r="E10" t="s">
-        <v>94</v>
-      </c>
-      <c r="F10" t="s">
-        <v>96</v>
-      </c>
-      <c r="G10" t="s">
-        <v>92</v>
-      </c>
-      <c r="H10" t="s">
-        <v>92</v>
-      </c>
-      <c r="I10" t="s">
-        <v>96</v>
-      </c>
-      <c r="J10" t="s">
-        <v>92</v>
-      </c>
-      <c r="K10" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -4419,29 +4419,29 @@
       <c r="C11">
         <v>1255</v>
       </c>
-      <c r="D11">
+      <c r="D11" t="s">
+        <v>94</v>
+      </c>
+      <c r="E11" t="s">
+        <v>92</v>
+      </c>
+      <c r="F11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G11" t="s">
+        <v>93</v>
+      </c>
+      <c r="H11" t="s">
+        <v>92</v>
+      </c>
+      <c r="I11" t="s">
+        <v>92</v>
+      </c>
+      <c r="J11" t="s">
+        <v>95</v>
+      </c>
+      <c r="K11">
         <v>17570</v>
-      </c>
-      <c r="E11" t="s">
-        <v>94</v>
-      </c>
-      <c r="F11" t="s">
-        <v>92</v>
-      </c>
-      <c r="G11" t="s">
-        <v>95</v>
-      </c>
-      <c r="H11" t="s">
-        <v>93</v>
-      </c>
-      <c r="I11" t="s">
-        <v>92</v>
-      </c>
-      <c r="J11" t="s">
-        <v>92</v>
-      </c>
-      <c r="K11" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -4454,29 +4454,29 @@
       <c r="C12">
         <v>1442</v>
       </c>
-      <c r="D12">
+      <c r="D12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E12" t="s">
+        <v>96</v>
+      </c>
+      <c r="F12" t="s">
+        <v>92</v>
+      </c>
+      <c r="G12" t="s">
+        <v>97</v>
+      </c>
+      <c r="H12" t="s">
+        <v>92</v>
+      </c>
+      <c r="I12" t="s">
+        <v>96</v>
+      </c>
+      <c r="J12" t="s">
+        <v>92</v>
+      </c>
+      <c r="K12">
         <v>20188</v>
-      </c>
-      <c r="E12" t="s">
-        <v>96</v>
-      </c>
-      <c r="F12" t="s">
-        <v>96</v>
-      </c>
-      <c r="G12" t="s">
-        <v>92</v>
-      </c>
-      <c r="H12" t="s">
-        <v>97</v>
-      </c>
-      <c r="I12" t="s">
-        <v>92</v>
-      </c>
-      <c r="J12" t="s">
-        <v>96</v>
-      </c>
-      <c r="K12" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -4489,29 +4489,29 @@
       <c r="C13">
         <v>1425</v>
       </c>
-      <c r="D13">
+      <c r="D13" t="s">
+        <v>96</v>
+      </c>
+      <c r="E13" t="s">
+        <v>96</v>
+      </c>
+      <c r="F13" t="s">
+        <v>92</v>
+      </c>
+      <c r="G13" t="s">
+        <v>92</v>
+      </c>
+      <c r="H13" t="s">
+        <v>97</v>
+      </c>
+      <c r="I13" t="s">
+        <v>92</v>
+      </c>
+      <c r="J13" t="s">
+        <v>95</v>
+      </c>
+      <c r="K13">
         <v>17100</v>
-      </c>
-      <c r="E13" t="s">
-        <v>96</v>
-      </c>
-      <c r="F13" t="s">
-        <v>96</v>
-      </c>
-      <c r="G13" t="s">
-        <v>92</v>
-      </c>
-      <c r="H13" t="s">
-        <v>92</v>
-      </c>
-      <c r="I13" t="s">
-        <v>97</v>
-      </c>
-      <c r="J13" t="s">
-        <v>92</v>
-      </c>
-      <c r="K13" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -4524,29 +4524,29 @@
       <c r="C14">
         <v>1244</v>
       </c>
-      <c r="D14">
+      <c r="D14" t="s">
+        <v>97</v>
+      </c>
+      <c r="E14" t="s">
+        <v>96</v>
+      </c>
+      <c r="F14" t="s">
+        <v>92</v>
+      </c>
+      <c r="G14" t="s">
+        <v>92</v>
+      </c>
+      <c r="H14" t="s">
+        <v>93</v>
+      </c>
+      <c r="I14" t="s">
+        <v>95</v>
+      </c>
+      <c r="J14" t="s">
+        <v>92</v>
+      </c>
+      <c r="K14">
         <v>14928</v>
-      </c>
-      <c r="E14" t="s">
-        <v>97</v>
-      </c>
-      <c r="F14" t="s">
-        <v>96</v>
-      </c>
-      <c r="G14" t="s">
-        <v>92</v>
-      </c>
-      <c r="H14" t="s">
-        <v>92</v>
-      </c>
-      <c r="I14" t="s">
-        <v>93</v>
-      </c>
-      <c r="J14" t="s">
-        <v>95</v>
-      </c>
-      <c r="K14" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -4559,29 +4559,29 @@
       <c r="C15">
         <v>1504</v>
       </c>
-      <c r="D15">
-        <v>15040</v>
+      <c r="D15" t="s">
+        <v>92</v>
       </c>
       <c r="E15" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="F15" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="G15" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="H15" t="s">
         <v>99</v>
       </c>
       <c r="I15" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="J15" t="s">
-        <v>92</v>
-      </c>
-      <c r="K15" t="s">
-        <v>96</v>
+        <v>96</v>
+      </c>
+      <c r="K15">
+        <v>15040</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -4594,29 +4594,29 @@
       <c r="C16">
         <v>1426</v>
       </c>
-      <c r="D16">
-        <v>14260</v>
+      <c r="D16" t="s">
+        <v>92</v>
       </c>
       <c r="E16" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="F16" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="G16" t="s">
+        <v>92</v>
+      </c>
+      <c r="H16" t="s">
         <v>94</v>
-      </c>
-      <c r="H16" t="s">
-        <v>92</v>
       </c>
       <c r="I16" t="s">
         <v>94</v>
       </c>
       <c r="J16" t="s">
-        <v>94</v>
-      </c>
-      <c r="K16" t="s">
-        <v>92</v>
+        <v>92</v>
+      </c>
+      <c r="K16">
+        <v>14260</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -4629,29 +4629,29 @@
       <c r="C17">
         <v>1164</v>
       </c>
-      <c r="D17">
+      <c r="D17" t="s">
+        <v>93</v>
+      </c>
+      <c r="E17" t="s">
+        <v>94</v>
+      </c>
+      <c r="F17" t="s">
+        <v>92</v>
+      </c>
+      <c r="G17" t="s">
+        <v>93</v>
+      </c>
+      <c r="H17" t="s">
+        <v>92</v>
+      </c>
+      <c r="I17" t="s">
+        <v>93</v>
+      </c>
+      <c r="J17" t="s">
+        <v>92</v>
+      </c>
+      <c r="K17">
         <v>10476</v>
-      </c>
-      <c r="E17" t="s">
-        <v>93</v>
-      </c>
-      <c r="F17" t="s">
-        <v>94</v>
-      </c>
-      <c r="G17" t="s">
-        <v>92</v>
-      </c>
-      <c r="H17" t="s">
-        <v>93</v>
-      </c>
-      <c r="I17" t="s">
-        <v>92</v>
-      </c>
-      <c r="J17" t="s">
-        <v>93</v>
-      </c>
-      <c r="K17" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -4664,29 +4664,29 @@
       <c r="C18">
         <v>1306</v>
       </c>
-      <c r="D18">
+      <c r="D18" t="s">
+        <v>92</v>
+      </c>
+      <c r="E18" t="s">
+        <v>100</v>
+      </c>
+      <c r="F18" t="s">
+        <v>96</v>
+      </c>
+      <c r="G18" t="s">
+        <v>92</v>
+      </c>
+      <c r="H18" t="s">
+        <v>96</v>
+      </c>
+      <c r="I18" t="s">
+        <v>93</v>
+      </c>
+      <c r="J18" t="s">
+        <v>92</v>
+      </c>
+      <c r="K18">
         <v>7836</v>
-      </c>
-      <c r="E18" t="s">
-        <v>92</v>
-      </c>
-      <c r="F18" t="s">
-        <v>100</v>
-      </c>
-      <c r="G18" t="s">
-        <v>96</v>
-      </c>
-      <c r="H18" t="s">
-        <v>92</v>
-      </c>
-      <c r="I18" t="s">
-        <v>96</v>
-      </c>
-      <c r="J18" t="s">
-        <v>93</v>
-      </c>
-      <c r="K18" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -4699,29 +4699,29 @@
       <c r="C19">
         <v>1154</v>
       </c>
-      <c r="D19">
+      <c r="D19" t="s">
+        <v>92</v>
+      </c>
+      <c r="E19" t="s">
+        <v>100</v>
+      </c>
+      <c r="F19" t="s">
+        <v>95</v>
+      </c>
+      <c r="G19" t="s">
+        <v>92</v>
+      </c>
+      <c r="H19" t="s">
+        <v>100</v>
+      </c>
+      <c r="I19" t="s">
+        <v>93</v>
+      </c>
+      <c r="J19" t="s">
+        <v>92</v>
+      </c>
+      <c r="K19">
         <v>6924</v>
-      </c>
-      <c r="E19" t="s">
-        <v>92</v>
-      </c>
-      <c r="F19" t="s">
-        <v>100</v>
-      </c>
-      <c r="G19" t="s">
-        <v>95</v>
-      </c>
-      <c r="H19" t="s">
-        <v>92</v>
-      </c>
-      <c r="I19" t="s">
-        <v>100</v>
-      </c>
-      <c r="J19" t="s">
-        <v>93</v>
-      </c>
-      <c r="K19" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -4734,29 +4734,29 @@
       <c r="C20">
         <v>1489</v>
       </c>
-      <c r="D20">
+      <c r="D20" t="s">
+        <v>93</v>
+      </c>
+      <c r="E20" t="s">
+        <v>92</v>
+      </c>
+      <c r="F20" t="s">
+        <v>92</v>
+      </c>
+      <c r="G20" t="s">
+        <v>96</v>
+      </c>
+      <c r="H20" t="s">
+        <v>94</v>
+      </c>
+      <c r="I20" t="s">
+        <v>92</v>
+      </c>
+      <c r="J20" t="s">
+        <v>94</v>
+      </c>
+      <c r="K20">
         <v>7445</v>
-      </c>
-      <c r="E20" t="s">
-        <v>93</v>
-      </c>
-      <c r="F20" t="s">
-        <v>92</v>
-      </c>
-      <c r="G20" t="s">
-        <v>92</v>
-      </c>
-      <c r="H20" t="s">
-        <v>96</v>
-      </c>
-      <c r="I20" t="s">
-        <v>94</v>
-      </c>
-      <c r="J20" t="s">
-        <v>92</v>
-      </c>
-      <c r="K20" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -4769,29 +4769,29 @@
       <c r="C21">
         <v>1408</v>
       </c>
-      <c r="D21">
+      <c r="D21" t="s">
+        <v>92</v>
+      </c>
+      <c r="E21" t="s">
+        <v>96</v>
+      </c>
+      <c r="F21" t="s">
+        <v>95</v>
+      </c>
+      <c r="G21" t="s">
+        <v>92</v>
+      </c>
+      <c r="H21" t="s">
+        <v>97</v>
+      </c>
+      <c r="I21" t="s">
+        <v>92</v>
+      </c>
+      <c r="J21" t="s">
+        <v>99</v>
+      </c>
+      <c r="K21">
         <v>5632</v>
-      </c>
-      <c r="E21" t="s">
-        <v>92</v>
-      </c>
-      <c r="F21" t="s">
-        <v>96</v>
-      </c>
-      <c r="G21" t="s">
-        <v>95</v>
-      </c>
-      <c r="H21" t="s">
-        <v>92</v>
-      </c>
-      <c r="I21" t="s">
-        <v>97</v>
-      </c>
-      <c r="J21" t="s">
-        <v>92</v>
-      </c>
-      <c r="K21" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -4804,29 +4804,29 @@
       <c r="C22">
         <v>1476</v>
       </c>
-      <c r="D22">
+      <c r="D22" t="s">
+        <v>95</v>
+      </c>
+      <c r="E22" t="s">
+        <v>96</v>
+      </c>
+      <c r="F22" t="s">
+        <v>92</v>
+      </c>
+      <c r="G22" t="s">
+        <v>96</v>
+      </c>
+      <c r="H22" t="s">
+        <v>92</v>
+      </c>
+      <c r="I22" t="s">
+        <v>92</v>
+      </c>
+      <c r="J22" t="s">
+        <v>96</v>
+      </c>
+      <c r="K22">
         <v>5904</v>
-      </c>
-      <c r="E22" t="s">
-        <v>95</v>
-      </c>
-      <c r="F22" t="s">
-        <v>96</v>
-      </c>
-      <c r="G22" t="s">
-        <v>92</v>
-      </c>
-      <c r="H22" t="s">
-        <v>96</v>
-      </c>
-      <c r="I22" t="s">
-        <v>92</v>
-      </c>
-      <c r="J22" t="s">
-        <v>92</v>
-      </c>
-      <c r="K22" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -4839,29 +4839,29 @@
       <c r="C23">
         <v>1294</v>
       </c>
-      <c r="D23">
+      <c r="D23" t="s">
+        <v>98</v>
+      </c>
+      <c r="E23" t="s">
+        <v>96</v>
+      </c>
+      <c r="F23" t="s">
+        <v>92</v>
+      </c>
+      <c r="G23" t="s">
+        <v>96</v>
+      </c>
+      <c r="H23" t="s">
+        <v>92</v>
+      </c>
+      <c r="I23" t="s">
+        <v>93</v>
+      </c>
+      <c r="J23" t="s">
+        <v>92</v>
+      </c>
+      <c r="K23">
         <v>5176</v>
-      </c>
-      <c r="E23" t="s">
-        <v>98</v>
-      </c>
-      <c r="F23" t="s">
-        <v>96</v>
-      </c>
-      <c r="G23" t="s">
-        <v>92</v>
-      </c>
-      <c r="H23" t="s">
-        <v>96</v>
-      </c>
-      <c r="I23" t="s">
-        <v>92</v>
-      </c>
-      <c r="J23" t="s">
-        <v>93</v>
-      </c>
-      <c r="K23" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -4874,29 +4874,29 @@
       <c r="C24">
         <v>1300</v>
       </c>
-      <c r="D24">
+      <c r="D24" t="s">
+        <v>99</v>
+      </c>
+      <c r="E24" t="s">
+        <v>94</v>
+      </c>
+      <c r="F24" t="s">
+        <v>92</v>
+      </c>
+      <c r="G24" t="s">
+        <v>99</v>
+      </c>
+      <c r="H24" t="s">
+        <v>92</v>
+      </c>
+      <c r="I24" t="s">
+        <v>93</v>
+      </c>
+      <c r="J24" t="s">
+        <v>92</v>
+      </c>
+      <c r="K24">
         <v>3900</v>
-      </c>
-      <c r="E24" t="s">
-        <v>99</v>
-      </c>
-      <c r="F24" t="s">
-        <v>94</v>
-      </c>
-      <c r="G24" t="s">
-        <v>92</v>
-      </c>
-      <c r="H24" t="s">
-        <v>99</v>
-      </c>
-      <c r="I24" t="s">
-        <v>92</v>
-      </c>
-      <c r="J24" t="s">
-        <v>93</v>
-      </c>
-      <c r="K24" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -4909,29 +4909,29 @@
       <c r="C25">
         <v>1266</v>
       </c>
-      <c r="D25">
+      <c r="D25" t="s">
+        <v>92</v>
+      </c>
+      <c r="E25" t="s">
+        <v>96</v>
+      </c>
+      <c r="F25" t="s">
+        <v>95</v>
+      </c>
+      <c r="G25" t="s">
+        <v>92</v>
+      </c>
+      <c r="H25" t="s">
+        <v>96</v>
+      </c>
+      <c r="I25" t="s">
+        <v>93</v>
+      </c>
+      <c r="J25" t="s">
+        <v>92</v>
+      </c>
+      <c r="K25">
         <v>3798</v>
-      </c>
-      <c r="E25" t="s">
-        <v>92</v>
-      </c>
-      <c r="F25" t="s">
-        <v>96</v>
-      </c>
-      <c r="G25" t="s">
-        <v>95</v>
-      </c>
-      <c r="H25" t="s">
-        <v>92</v>
-      </c>
-      <c r="I25" t="s">
-        <v>96</v>
-      </c>
-      <c r="J25" t="s">
-        <v>93</v>
-      </c>
-      <c r="K25" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -4944,29 +4944,29 @@
       <c r="C26">
         <v>1405</v>
       </c>
-      <c r="D26">
+      <c r="D26" t="s">
+        <v>92</v>
+      </c>
+      <c r="E26" t="s">
+        <v>100</v>
+      </c>
+      <c r="F26" t="s">
+        <v>92</v>
+      </c>
+      <c r="G26" t="s">
+        <v>97</v>
+      </c>
+      <c r="H26" t="s">
+        <v>93</v>
+      </c>
+      <c r="I26" t="s">
+        <v>92</v>
+      </c>
+      <c r="J26" t="s">
+        <v>94</v>
+      </c>
+      <c r="K26">
         <v>4215</v>
-      </c>
-      <c r="E26" t="s">
-        <v>92</v>
-      </c>
-      <c r="F26" t="s">
-        <v>100</v>
-      </c>
-      <c r="G26" t="s">
-        <v>92</v>
-      </c>
-      <c r="H26" t="s">
-        <v>97</v>
-      </c>
-      <c r="I26" t="s">
-        <v>93</v>
-      </c>
-      <c r="J26" t="s">
-        <v>92</v>
-      </c>
-      <c r="K26" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -4979,29 +4979,29 @@
       <c r="C27">
         <v>1428</v>
       </c>
-      <c r="D27">
+      <c r="D27" t="s">
+        <v>93</v>
+      </c>
+      <c r="E27" t="s">
+        <v>92</v>
+      </c>
+      <c r="F27" t="s">
+        <v>96</v>
+      </c>
+      <c r="G27" t="s">
+        <v>92</v>
+      </c>
+      <c r="H27" t="s">
+        <v>97</v>
+      </c>
+      <c r="I27" t="s">
+        <v>92</v>
+      </c>
+      <c r="J27" t="s">
+        <v>97</v>
+      </c>
+      <c r="K27">
         <v>4284</v>
-      </c>
-      <c r="E27" t="s">
-        <v>93</v>
-      </c>
-      <c r="F27" t="s">
-        <v>92</v>
-      </c>
-      <c r="G27" t="s">
-        <v>96</v>
-      </c>
-      <c r="H27" t="s">
-        <v>92</v>
-      </c>
-      <c r="I27" t="s">
-        <v>97</v>
-      </c>
-      <c r="J27" t="s">
-        <v>92</v>
-      </c>
-      <c r="K27" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="28" spans="1:11">
@@ -5014,29 +5014,29 @@
       <c r="C28">
         <v>1436</v>
       </c>
-      <c r="D28">
+      <c r="D28" t="s">
+        <v>96</v>
+      </c>
+      <c r="E28" t="s">
+        <v>92</v>
+      </c>
+      <c r="F28" t="s">
+        <v>96</v>
+      </c>
+      <c r="G28" t="s">
+        <v>99</v>
+      </c>
+      <c r="H28" t="s">
+        <v>92</v>
+      </c>
+      <c r="I28" t="s">
+        <v>94</v>
+      </c>
+      <c r="J28" t="s">
+        <v>92</v>
+      </c>
+      <c r="K28">
         <v>2872</v>
-      </c>
-      <c r="E28" t="s">
-        <v>96</v>
-      </c>
-      <c r="F28" t="s">
-        <v>92</v>
-      </c>
-      <c r="G28" t="s">
-        <v>96</v>
-      </c>
-      <c r="H28" t="s">
-        <v>99</v>
-      </c>
-      <c r="I28" t="s">
-        <v>92</v>
-      </c>
-      <c r="J28" t="s">
-        <v>94</v>
-      </c>
-      <c r="K28" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="29" spans="1:11">
@@ -5049,29 +5049,29 @@
       <c r="C29">
         <v>1298</v>
       </c>
-      <c r="D29">
+      <c r="D29" t="s">
+        <v>93</v>
+      </c>
+      <c r="E29" t="s">
+        <v>92</v>
+      </c>
+      <c r="F29" t="s">
+        <v>92</v>
+      </c>
+      <c r="G29" t="s">
+        <v>99</v>
+      </c>
+      <c r="H29" t="s">
+        <v>96</v>
+      </c>
+      <c r="I29" t="s">
+        <v>92</v>
+      </c>
+      <c r="J29" t="s">
+        <v>93</v>
+      </c>
+      <c r="K29">
         <v>2596</v>
-      </c>
-      <c r="E29" t="s">
-        <v>93</v>
-      </c>
-      <c r="F29" t="s">
-        <v>92</v>
-      </c>
-      <c r="G29" t="s">
-        <v>92</v>
-      </c>
-      <c r="H29" t="s">
-        <v>99</v>
-      </c>
-      <c r="I29" t="s">
-        <v>96</v>
-      </c>
-      <c r="J29" t="s">
-        <v>92</v>
-      </c>
-      <c r="K29" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="30" spans="1:11">
@@ -5084,29 +5084,29 @@
       <c r="C30">
         <v>1260</v>
       </c>
-      <c r="D30">
+      <c r="D30" t="s">
+        <v>96</v>
+      </c>
+      <c r="E30" t="s">
+        <v>93</v>
+      </c>
+      <c r="F30" t="s">
+        <v>92</v>
+      </c>
+      <c r="G30" t="s">
+        <v>96</v>
+      </c>
+      <c r="H30" t="s">
+        <v>92</v>
+      </c>
+      <c r="I30" t="s">
+        <v>93</v>
+      </c>
+      <c r="J30" t="s">
+        <v>92</v>
+      </c>
+      <c r="K30">
         <v>2520</v>
-      </c>
-      <c r="E30" t="s">
-        <v>96</v>
-      </c>
-      <c r="F30" t="s">
-        <v>93</v>
-      </c>
-      <c r="G30" t="s">
-        <v>92</v>
-      </c>
-      <c r="H30" t="s">
-        <v>96</v>
-      </c>
-      <c r="I30" t="s">
-        <v>92</v>
-      </c>
-      <c r="J30" t="s">
-        <v>93</v>
-      </c>
-      <c r="K30" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -5119,29 +5119,29 @@
       <c r="C31">
         <v>1356</v>
       </c>
-      <c r="D31">
+      <c r="D31" t="s">
+        <v>92</v>
+      </c>
+      <c r="E31" t="s">
+        <v>100</v>
+      </c>
+      <c r="F31" t="s">
+        <v>92</v>
+      </c>
+      <c r="G31" t="s">
+        <v>96</v>
+      </c>
+      <c r="H31" t="s">
+        <v>97</v>
+      </c>
+      <c r="I31" t="s">
+        <v>92</v>
+      </c>
+      <c r="J31" t="s">
+        <v>93</v>
+      </c>
+      <c r="K31">
         <v>1356</v>
-      </c>
-      <c r="E31" t="s">
-        <v>92</v>
-      </c>
-      <c r="F31" t="s">
-        <v>100</v>
-      </c>
-      <c r="G31" t="s">
-        <v>92</v>
-      </c>
-      <c r="H31" t="s">
-        <v>96</v>
-      </c>
-      <c r="I31" t="s">
-        <v>97</v>
-      </c>
-      <c r="J31" t="s">
-        <v>92</v>
-      </c>
-      <c r="K31" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -5154,29 +5154,29 @@
       <c r="C32">
         <v>1591</v>
       </c>
-      <c r="D32">
+      <c r="D32" t="s">
+        <v>96</v>
+      </c>
+      <c r="E32" t="s">
+        <v>94</v>
+      </c>
+      <c r="F32" t="s">
+        <v>92</v>
+      </c>
+      <c r="G32" t="s">
+        <v>92</v>
+      </c>
+      <c r="H32" t="s">
+        <v>96</v>
+      </c>
+      <c r="I32" t="s">
+        <v>92</v>
+      </c>
+      <c r="J32" t="s">
+        <v>94</v>
+      </c>
+      <c r="K32">
         <v>1591</v>
-      </c>
-      <c r="E32" t="s">
-        <v>96</v>
-      </c>
-      <c r="F32" t="s">
-        <v>94</v>
-      </c>
-      <c r="G32" t="s">
-        <v>92</v>
-      </c>
-      <c r="H32" t="s">
-        <v>92</v>
-      </c>
-      <c r="I32" t="s">
-        <v>96</v>
-      </c>
-      <c r="J32" t="s">
-        <v>92</v>
-      </c>
-      <c r="K32" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="33" spans="1:11">
@@ -5189,29 +5189,29 @@
       <c r="C33">
         <v>1448</v>
       </c>
-      <c r="D33">
+      <c r="D33" t="s">
+        <v>97</v>
+      </c>
+      <c r="E33" t="s">
+        <v>92</v>
+      </c>
+      <c r="F33" t="s">
+        <v>94</v>
+      </c>
+      <c r="G33" t="s">
+        <v>96</v>
+      </c>
+      <c r="H33" t="s">
+        <v>92</v>
+      </c>
+      <c r="I33" t="s">
+        <v>96</v>
+      </c>
+      <c r="J33" t="s">
+        <v>92</v>
+      </c>
+      <c r="K33">
         <v>1448</v>
-      </c>
-      <c r="E33" t="s">
-        <v>97</v>
-      </c>
-      <c r="F33" t="s">
-        <v>92</v>
-      </c>
-      <c r="G33" t="s">
-        <v>94</v>
-      </c>
-      <c r="H33" t="s">
-        <v>96</v>
-      </c>
-      <c r="I33" t="s">
-        <v>92</v>
-      </c>
-      <c r="J33" t="s">
-        <v>96</v>
-      </c>
-      <c r="K33" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="34" spans="1:11">
@@ -5224,29 +5224,29 @@
       <c r="C34">
         <v>1364</v>
       </c>
-      <c r="D34">
+      <c r="D34" t="s">
+        <v>97</v>
+      </c>
+      <c r="E34" t="s">
+        <v>100</v>
+      </c>
+      <c r="F34" t="s">
+        <v>92</v>
+      </c>
+      <c r="G34" t="s">
+        <v>92</v>
+      </c>
+      <c r="H34" t="s">
+        <v>97</v>
+      </c>
+      <c r="I34" t="s">
+        <v>96</v>
+      </c>
+      <c r="J34" t="s">
+        <v>92</v>
+      </c>
+      <c r="K34">
         <v>1364</v>
-      </c>
-      <c r="E34" t="s">
-        <v>97</v>
-      </c>
-      <c r="F34" t="s">
-        <v>100</v>
-      </c>
-      <c r="G34" t="s">
-        <v>92</v>
-      </c>
-      <c r="H34" t="s">
-        <v>92</v>
-      </c>
-      <c r="I34" t="s">
-        <v>97</v>
-      </c>
-      <c r="J34" t="s">
-        <v>96</v>
-      </c>
-      <c r="K34" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="35" spans="1:11">
@@ -5259,29 +5259,29 @@
       <c r="C35">
         <v>1368</v>
       </c>
-      <c r="D35">
+      <c r="D35" t="s">
+        <v>96</v>
+      </c>
+      <c r="E35" t="s">
+        <v>93</v>
+      </c>
+      <c r="F35" t="s">
+        <v>92</v>
+      </c>
+      <c r="G35" t="s">
+        <v>92</v>
+      </c>
+      <c r="H35" t="s">
+        <v>93</v>
+      </c>
+      <c r="I35" t="s">
+        <v>92</v>
+      </c>
+      <c r="J35" t="s">
+        <v>96</v>
+      </c>
+      <c r="K35">
         <v>1368</v>
-      </c>
-      <c r="E35" t="s">
-        <v>96</v>
-      </c>
-      <c r="F35" t="s">
-        <v>93</v>
-      </c>
-      <c r="G35" t="s">
-        <v>92</v>
-      </c>
-      <c r="H35" t="s">
-        <v>92</v>
-      </c>
-      <c r="I35" t="s">
-        <v>93</v>
-      </c>
-      <c r="J35" t="s">
-        <v>92</v>
-      </c>
-      <c r="K35" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -5294,29 +5294,29 @@
       <c r="C36">
         <v>1266</v>
       </c>
-      <c r="D36">
+      <c r="D36" t="s">
+        <v>92</v>
+      </c>
+      <c r="E36" t="s">
+        <v>93</v>
+      </c>
+      <c r="F36" t="s">
+        <v>93</v>
+      </c>
+      <c r="G36" t="s">
+        <v>92</v>
+      </c>
+      <c r="H36" t="s">
+        <v>96</v>
+      </c>
+      <c r="I36" t="s">
+        <v>94</v>
+      </c>
+      <c r="J36" t="s">
+        <v>92</v>
+      </c>
+      <c r="K36">
         <v>1266</v>
-      </c>
-      <c r="E36" t="s">
-        <v>92</v>
-      </c>
-      <c r="F36" t="s">
-        <v>93</v>
-      </c>
-      <c r="G36" t="s">
-        <v>93</v>
-      </c>
-      <c r="H36" t="s">
-        <v>92</v>
-      </c>
-      <c r="I36" t="s">
-        <v>96</v>
-      </c>
-      <c r="J36" t="s">
-        <v>94</v>
-      </c>
-      <c r="K36" t="s">
-        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>